<commit_message>
Fixed upload of wrong BOM file
</commit_message>
<xml_diff>
--- a/BOM-revised.xlsx
+++ b/BOM-revised.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Nemo\Dropbox\Shaker\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B099E32F-28A9-4FCB-A6CF-24CB6908D920}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93DF347B-3505-42A8-ADFE-953E0BF34153}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="23236" windowHeight="13875" xr2:uid="{162B4DA1-8CE5-452B-909C-5598A1AF88A8}"/>
+    <workbookView xWindow="6735" yWindow="3548" windowWidth="18833" windowHeight="12254" xr2:uid="{162B4DA1-8CE5-452B-909C-5598A1AF88A8}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
   <si>
     <t>Item</t>
   </si>
@@ -86,50 +86,45 @@
     <t>https://www.amazon.com/ELEGOO-Board-ATmega328P-ATMEGA16U2-Compliant/dp/B01EWOE0UU/ref=sr_1_2_sspa?crid=2MVA27AWSN0Q0&amp;dib=eyJ2IjoiMSJ9.XbKE6b0NGJdls38suMJhLXJd6g6Vup0nHHmmYI4Zo9rRaTJjfJhh9u9oYVUHTxDJ6SKxHRlTaj_vlmAHzN3FPHtbdYeIWy2us3Il6HYOTXlj3zNZvmq8CJW2Vj2onUr2FivGdnr6sM4cs_6uKW2BOZHbN6KdgU8Sdhvv44XseCd8RrgxiYhAcXd_SSu9UqZQchXXr7dWF0djXiEWddNBiRZHuulwUBnHNt9ajREK2X4.vfHKXD0BHtrR_6xbwolCcY_EoXDMBtATR0Ngyys9sJU&amp;dib_tag=se&amp;keywords=arduino+uno&amp;qid=1709933235&amp;sprefix=arduino+uno%2Caps%2C85&amp;sr=8-2-spons&amp;sp_csd=d2lkZ2V0TmFtZT1zcF9hdGY&amp;psc=1</t>
   </si>
   <si>
-    <t>Plywood (base+table)</t>
-  </si>
-  <si>
-    <t>Estimate</t>
-  </si>
-  <si>
     <t>PETG Fillament - gray 2 pack</t>
   </si>
   <si>
     <t>https://us.store.bambulab.com/products/petg-basic?variant=41184283852936</t>
   </si>
   <si>
-    <t>TPU Fillament - red</t>
-  </si>
-  <si>
-    <t>https://www.amazon.com/Overture-Filament-Flexible-Consumables-Dimensional/dp/B07VBL6XHH/ref=sr_1_1_sspa?crid=1MBN2HQVDSJ2Y&amp;dib=eyJ2IjoiMSJ9.xVB8WRC28bs6U8XSXGdY-ei5Rclu2VTLJcxjWhGsnTrrV9ZCDMEACi2ggyJFUhFhJ3WiPBmXcUBdZN3PhZhr8sF0VxOiyS_IzpPi33dozHUK8uXlr8XSWsJ3pvVomDUhA9UpQzVpGWrbHVuQsgWTs-uWR52ELNs67zeCCHp6PpxCM8D-719u0EzGXDJ1lkYpwd7VjCF37m_rPt8Y5UM3JbEBzbRrAtpceR-qmVkgJnM.kvHMOMtIWZ11ECqYNDQ0IK0u4ciRv6mZKGZBwSdRnoI&amp;dib_tag=se&amp;keywords=overture%2Btpu&amp;qid=1709932972&amp;sprefix=overture%2Btpu%2Caps%2C113&amp;sr=8-1-spons&amp;sp_csd=d2lkZ2V0TmFtZT1zcF9hdGY&amp;th=1</t>
-  </si>
-  <si>
-    <t>Rotary Encoders</t>
-  </si>
-  <si>
-    <t>https://www.amazon.com/WayinTop-Degree-Encoder-Development-Arduino/dp/B07T3672VK/ref=sr_1_2?crid=2WA0K3F8DUTF4&amp;dib=eyJ2IjoiMSJ9.fbZwo1EdB-FxvnxRUw6gmtggfJzYR2n1R0cYU6NUd0TxBE1wOyhoQIyqcISe5_90pS5gUUz1JKcvbvos8CME2AfZRSmsfr3h6BfSA-RNIT_BPM0Xq2TtnbqdjSz990vE0I-qIWLzuuCV1F2t_iyJQeUuC76BOHLw6uoRPwA5AHz8YeDqrV5aQIiscW17YzhwAu08HLNR86TLjJnXt-Spc8eE3uW-OgceQjUaF5VpZNw.nP7F7MStSDPxuhEVrjA7lWBxNdx8YhIZ1YD3zE48Ztk&amp;dib_tag=se&amp;keywords=arduino+encoders&amp;qid=1708031441&amp;sprefix=arduino+encoders%2Caps%2C77&amp;sr=8-2</t>
-  </si>
-  <si>
-    <t>Hardened Steel Nozzle</t>
-  </si>
-  <si>
-    <t>https://us.store.bambulab.com/products/complete-hotend-assembly-p1p</t>
-  </si>
-  <si>
-    <t>Hardened Steel Gearset</t>
-  </si>
-  <si>
-    <t>https://us.store.bambulab.com/products/hardened-steel-extruder-gear-assembly?variant=40983091904648</t>
+    <t>https://www.amazon.com/S-360-24-Switch-Transformer-Supply-Switching/dp/B0DFB84KWL</t>
+  </si>
+  <si>
+    <t>S-360-24 Power Supply</t>
+  </si>
+  <si>
+    <t>Stepper motor driver</t>
+  </si>
+  <si>
+    <t>https://www.amazon.com/gp/product/B07HHS14VQ/ref=ox_sc_saved_title_4?smid=A1RTFVCI20VZT2&amp;th=1</t>
+  </si>
+  <si>
+    <t>Power supply cable</t>
+  </si>
+  <si>
+    <t>https://www.amazon.com/Pinfox-Universal-Appliance-Replacement-Pigtail/dp/B06XQZFD36?psc=1&amp;pd_rd_w=b7wV9&amp;content-id=amzn1.sym.ea1d9533-fbb7-4608-bb6f-bfdceb6f6336&amp;pf_rd_p=ea1d9533-fbb7-4608-bb6f-bfdceb6f6336&amp;pf_rd_r=Q0F12MRDFC97FFS67FJN&amp;pd_rd_wg=WmgqK&amp;pd_rd_r=7c7c2440-dd90-4c5f-8149-85fe80e55bb4&amp;ref_=sspa_dk_detail_2</t>
+  </si>
+  <si>
+    <t>Jumper Wires</t>
+  </si>
+  <si>
+    <t>https://www.amazon.com/Elegoo-EL-CP-004-Multicolored-Breadboard-arduino/dp/B01EV70C78/ref=sr_1_1_sspa?crid=3AYWNBM1IKLQK&amp;dib=eyJ2IjoiMSJ9.qJE7UjNibAzbwpMmx2tJ0wsODsLFmAeWjM_Y5uH3tYd4xWxyTvRSv87TMwvZNDUGaZ84Bx3QSEUrcEsivgesT8TAPAYRlnMB6tGewY-1N1Y7m8m7t75Gp5Mmcd32mwtnh3rv9ZbjtNpwnLidFh24BMgayt2ypyEtyVn6FCthQ-EHtRzAMDEqw5q68NfKPwLRh2pauKij0zNfk0xXul2W16LurHvGHwAsCm8UGPESSQs.6TtV5nH-YCbfjCVUKk2BbRzz8dECqLgGtGDFvil3UsQ&amp;dib_tag=se&amp;keywords=hobby+jumper+wires&amp;qid=1727365183&amp;sprefix=hobby+jumper+wires%2Caps%2C86&amp;sr=8-1-spons&amp;sp_csd=d2lkZ2V0TmFtZT1zcF9hdGY&amp;psc=1</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
+    <numFmt numFmtId="8" formatCode="&quot;$&quot;#,##0.00_);[Red]\(&quot;$&quot;#,##0.00\)"/>
     <numFmt numFmtId="164" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -153,8 +148,15 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -173,6 +175,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC0E4F5"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="12">
     <border>
@@ -318,7 +326,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -353,6 +361,11 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="8" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="1" applyFill="1"/>
+    <xf numFmtId="8" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -738,7 +751,7 @@
       </c>
       <c r="H3" s="11">
         <f>SUM(F3:F35)</f>
-        <v>249.89000000000001</v>
+        <v>186.38</v>
       </c>
     </row>
     <row r="4" spans="2:8" x14ac:dyDescent="0.45">
@@ -821,30 +834,30 @@
     </row>
     <row r="8" spans="2:8" x14ac:dyDescent="0.45">
       <c r="B8" s="12" t="s">
-        <v>16</v>
-      </c>
-      <c r="C8" s="17" t="s">
-        <v>17</v>
+        <v>19</v>
+      </c>
+      <c r="C8" s="21" t="s">
+        <v>18</v>
       </c>
       <c r="D8" s="14">
-        <v>20</v>
+        <v>22.5</v>
       </c>
       <c r="E8" s="15">
         <v>1</v>
       </c>
       <c r="F8" s="16">
         <f t="shared" si="0"/>
-        <v>20</v>
+        <v>22.5</v>
       </c>
       <c r="G8" s="17"/>
       <c r="H8" s="18"/>
     </row>
     <row r="9" spans="2:8" x14ac:dyDescent="0.45">
       <c r="B9" s="6" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C9" s="19" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="D9" s="8">
         <v>27.99</v>
@@ -859,81 +872,70 @@
       <c r="H9" s="20"/>
     </row>
     <row r="10" spans="2:8" x14ac:dyDescent="0.45">
-      <c r="B10" s="12" t="s">
+      <c r="B10" s="28" t="s">
         <v>20</v>
       </c>
-      <c r="C10" s="21" t="s">
+      <c r="C10" s="19" t="s">
         <v>21</v>
       </c>
-      <c r="D10" s="14">
-        <v>28.99</v>
+      <c r="D10" s="29">
+        <v>9.98</v>
       </c>
       <c r="E10" s="15">
         <v>1</v>
       </c>
       <c r="F10" s="16">
         <f t="shared" si="0"/>
-        <v>28.99</v>
+        <v>9.98</v>
       </c>
       <c r="G10" s="17"/>
       <c r="H10" s="18"/>
     </row>
     <row r="11" spans="2:8" x14ac:dyDescent="0.45">
-      <c r="B11" s="6" t="s">
+      <c r="B11" s="28" t="s">
         <v>22</v>
       </c>
       <c r="C11" s="19" t="s">
         <v>23</v>
       </c>
-      <c r="D11" s="8">
-        <v>11.99</v>
-      </c>
-      <c r="E11" s="9">
+      <c r="D11" s="29">
+        <v>12.99</v>
+      </c>
+      <c r="E11" s="15">
         <v>1</v>
       </c>
-      <c r="F11" s="10">
-        <f t="shared" si="0"/>
-        <v>11.99</v>
+      <c r="F11" s="16">
+        <f t="shared" ref="F11:F13" si="1">(D11*E11)</f>
+        <v>12.99</v>
       </c>
       <c r="H11" s="20"/>
     </row>
     <row r="12" spans="2:8" x14ac:dyDescent="0.45">
-      <c r="B12" s="12" t="s">
+      <c r="B12" s="28" t="s">
         <v>24</v>
       </c>
-      <c r="C12" s="21" t="s">
+      <c r="C12" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="D12" s="14">
-        <v>34.99</v>
+      <c r="D12" s="29">
+        <v>6.98</v>
       </c>
       <c r="E12" s="15">
         <v>1</v>
       </c>
       <c r="F12" s="16">
-        <f t="shared" si="0"/>
-        <v>34.99</v>
+        <f t="shared" si="1"/>
+        <v>6.98</v>
       </c>
       <c r="G12" s="17"/>
       <c r="H12" s="18"/>
     </row>
     <row r="13" spans="2:8" x14ac:dyDescent="0.45">
-      <c r="B13" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="C13" s="19" t="s">
-        <v>27</v>
-      </c>
-      <c r="D13" s="8">
-        <v>19.989999999999998</v>
-      </c>
-      <c r="E13" s="9">
-        <v>1</v>
-      </c>
-      <c r="F13" s="10">
-        <f t="shared" si="0"/>
-        <v>19.989999999999998</v>
-      </c>
+      <c r="B13" s="30"/>
+      <c r="C13" s="31"/>
+      <c r="D13" s="32"/>
+      <c r="E13" s="15"/>
+      <c r="F13" s="16"/>
       <c r="H13" s="20"/>
     </row>
     <row r="14" spans="2:8" x14ac:dyDescent="0.45">
@@ -1186,12 +1188,12 @@
     <hyperlink ref="C4" r:id="rId2" xr:uid="{91ED1588-1F31-4E66-B37C-24CD0D538938}"/>
     <hyperlink ref="C6" r:id="rId3" display="https://www.amazon.com/Stepper-57x57x113mm-Stepping-23HS2430B-Engraving/dp/B0CQLJJ2K2/ref=sr_1_1?crid=YWSF9T3E282K&amp;keywords=nema%2Bstepper%2Bmotor&amp;qid=1707849890&amp;s=industrial&amp;sprefix=nema%2Bstepper%2Bmotor%2Cindustrial%2C298&amp;sr=1-1-spons&amp;sp_csd=d2lkZ2V0TmFtZT1zcF9hdGY&amp;th=1" xr:uid="{C69A6F61-BDBA-402D-B91C-F83C73C0E8AB}"/>
     <hyperlink ref="C7" r:id="rId4" display="https://www.amazon.com/ELEGOO-Board-ATmega328P-ATMEGA16U2-Compliant/dp/B01EWOE0UU/ref=sr_1_2_sspa?crid=2MVA27AWSN0Q0&amp;dib=eyJ2IjoiMSJ9.XbKE6b0NGJdls38suMJhLXJd6g6Vup0nHHmmYI4Zo9rRaTJjfJhh9u9oYVUHTxDJ6SKxHRlTaj_vlmAHzN3FPHtbdYeIWy2us3Il6HYOTXlj3zNZvmq8CJW2Vj2onUr2FivGdnr6sM4cs_6uKW2BOZHbN6KdgU8Sdhvv44XseCd8RrgxiYhAcXd_SSu9UqZQchXXr7dWF0djXiEWddNBiRZHuulwUBnHNt9ajREK2X4.vfHKXD0BHtrR_6xbwolCcY_EoXDMBtATR0Ngyys9sJU&amp;dib_tag=se&amp;keywords=arduino+uno&amp;qid=1709933235&amp;sprefix=arduino+uno%2Caps%2C85&amp;sr=8-2-spons&amp;sp_csd=d2lkZ2V0TmFtZT1zcF9hdGY&amp;psc=1" xr:uid="{C8E8E90A-0972-4B17-9B5E-E7A025EFD89D}"/>
-    <hyperlink ref="C10" r:id="rId5" display="https://www.amazon.com/Overture-Filament-Flexible-Consumables-Dimensional/dp/B07VBL6XHH/ref=sr_1_1_sspa?crid=1MBN2HQVDSJ2Y&amp;dib=eyJ2IjoiMSJ9.xVB8WRC28bs6U8XSXGdY-ei5Rclu2VTLJcxjWhGsnTrrV9ZCDMEACi2ggyJFUhFhJ3WiPBmXcUBdZN3PhZhr8sF0VxOiyS_IzpPi33dozHUK8uXlr8XSWsJ3pvVomDUhA9UpQzVpGWrbHVuQsgWTs-uWR52ELNs67zeCCHp6PpxCM8D-719u0EzGXDJ1lkYpwd7VjCF37m_rPt8Y5UM3JbEBzbRrAtpceR-qmVkgJnM.kvHMOMtIWZ11ECqYNDQ0IK0u4ciRv6mZKGZBwSdRnoI&amp;dib_tag=se&amp;keywords=overture%2Btpu&amp;qid=1709932972&amp;sprefix=overture%2Btpu%2Caps%2C113&amp;sr=8-1-spons&amp;sp_csd=d2lkZ2V0TmFtZT1zcF9hdGY&amp;th=1" xr:uid="{F6C0BC89-9119-46A6-86AA-AF61FD11CD56}"/>
-    <hyperlink ref="C11" r:id="rId6" display="https://www.amazon.com/WayinTop-Degree-Encoder-Development-Arduino/dp/B07T3672VK/ref=sr_1_2?crid=2WA0K3F8DUTF4&amp;dib=eyJ2IjoiMSJ9.fbZwo1EdB-FxvnxRUw6gmtggfJzYR2n1R0cYU6NUd0TxBE1wOyhoQIyqcISe5_90pS5gUUz1JKcvbvos8CME2AfZRSmsfr3h6BfSA-RNIT_BPM0Xq2TtnbqdjSz990vE0I-qIWLzuuCV1F2t_iyJQeUuC76BOHLw6uoRPwA5AHz8YeDqrV5aQIiscW17YzhwAu08HLNR86TLjJnXt-Spc8eE3uW-OgceQjUaF5VpZNw.nP7F7MStSDPxuhEVrjA7lWBxNdx8YhIZ1YD3zE48Ztk&amp;dib_tag=se&amp;keywords=arduino+encoders&amp;qid=1708031441&amp;sprefix=arduino+encoders%2Caps%2C77&amp;sr=8-2" xr:uid="{CC99F62C-75DA-4262-8D29-D4050395BDBC}"/>
-    <hyperlink ref="C9" r:id="rId7" xr:uid="{C2852DC2-2D79-4731-BBEC-7BBD3E2BCFEC}"/>
-    <hyperlink ref="C5" r:id="rId8" display="https://www.amazon.com/Zeelo-Timing-Pulley-Meters-Printer/dp/B08SMFM3Z6/ref=sr_1_4?crid=5CPTEARD86FW&amp;dib=eyJ2IjoiMSJ9.tiebSJUcXdPWycpTXDsZ3UTQsMh6AraeLngnxIhhgKclt8Ey7OacIRAp7gbs9aKIqnE4R3THNIy1FuyczSKLw3S2IgKhpi_wsAl-eMHp7dAJTepVaQvYQM4lH1w7x6GLhMGb7JpW8X3csTwS2mDp6Ud7I_bstAXP-3Aex9PoGwFKjUPKeLzODqX0LvqoA-05H9N2jdJ1FwbZijA7fLPDNNou6yxVkAx8-ft1lD5ZhKM.ZFciUQEe0h5qqczGcxncQr9_i2s0DDp7qcC4UDw5wNc&amp;dib_tag=se&amp;keywords=timing%2Bbelt%2Bfor%2Bnema&amp;qid=1709750668&amp;sprefix=timing%2Bbelt%2Bfor%2Bnema%2Caps%2C87&amp;sr=8-4&amp;th=1" xr:uid="{595A8D42-CA18-4100-9AC2-85195D587E6D}"/>
-    <hyperlink ref="C12" r:id="rId9" xr:uid="{DF239D0A-CA48-4C56-9480-CF9DFDA6B8E9}"/>
-    <hyperlink ref="C13" r:id="rId10" xr:uid="{ABE90DE0-15DB-46AD-BC94-9D2C4119C0EE}"/>
+    <hyperlink ref="C9" r:id="rId5" xr:uid="{C2852DC2-2D79-4731-BBEC-7BBD3E2BCFEC}"/>
+    <hyperlink ref="C5" r:id="rId6" display="https://www.amazon.com/Zeelo-Timing-Pulley-Meters-Printer/dp/B08SMFM3Z6/ref=sr_1_4?crid=5CPTEARD86FW&amp;dib=eyJ2IjoiMSJ9.tiebSJUcXdPWycpTXDsZ3UTQsMh6AraeLngnxIhhgKclt8Ey7OacIRAp7gbs9aKIqnE4R3THNIy1FuyczSKLw3S2IgKhpi_wsAl-eMHp7dAJTepVaQvYQM4lH1w7x6GLhMGb7JpW8X3csTwS2mDp6Ud7I_bstAXP-3Aex9PoGwFKjUPKeLzODqX0LvqoA-05H9N2jdJ1FwbZijA7fLPDNNou6yxVkAx8-ft1lD5ZhKM.ZFciUQEe0h5qqczGcxncQr9_i2s0DDp7qcC4UDw5wNc&amp;dib_tag=se&amp;keywords=timing%2Bbelt%2Bfor%2Bnema&amp;qid=1709750668&amp;sprefix=timing%2Bbelt%2Bfor%2Bnema%2Caps%2C87&amp;sr=8-4&amp;th=1" xr:uid="{595A8D42-CA18-4100-9AC2-85195D587E6D}"/>
+    <hyperlink ref="C8" r:id="rId7" xr:uid="{EE957A94-ADFC-4464-A090-497525A7A4E9}"/>
+    <hyperlink ref="C10" r:id="rId8" xr:uid="{3753890B-115D-499D-9F9A-4556DD8E68CA}"/>
+    <hyperlink ref="C11" r:id="rId9" display="https://www.amazon.com/Pinfox-Universal-Appliance-Replacement-Pigtail/dp/B06XQZFD36?psc=1&amp;pd_rd_w=b7wV9&amp;content-id=amzn1.sym.ea1d9533-fbb7-4608-bb6f-bfdceb6f6336&amp;pf_rd_p=ea1d9533-fbb7-4608-bb6f-bfdceb6f6336&amp;pf_rd_r=Q0F12MRDFC97FFS67FJN&amp;pd_rd_wg=WmgqK&amp;pd_rd_r=7c7c2440-dd90-4c5f-8149-85fe80e55bb4&amp;ref_=sspa_dk_detail_2" xr:uid="{793702DD-9135-4BDC-8F11-969742E47FBC}"/>
+    <hyperlink ref="C12" r:id="rId10" display="https://www.amazon.com/Elegoo-EL-CP-004-Multicolored-Breadboard-arduino/dp/B01EV70C78/ref=sr_1_1_sspa?crid=3AYWNBM1IKLQK&amp;dib=eyJ2IjoiMSJ9.qJE7UjNibAzbwpMmx2tJ0wsODsLFmAeWjM_Y5uH3tYd4xWxyTvRSv87TMwvZNDUGaZ84Bx3QSEUrcEsivgesT8TAPAYRlnMB6tGewY-1N1Y7m8m7t75Gp5Mmcd32mwtnh3rv9ZbjtNpwnLidFh24BMgayt2ypyEtyVn6FCthQ-EHtRzAMDEqw5q68NfKPwLRh2pauKij0zNfk0xXul2W16LurHvGHwAsCm8UGPESSQs.6TtV5nH-YCbfjCVUKk2BbRzz8dECqLgGtGDFvil3UsQ&amp;dib_tag=se&amp;keywords=hobby+jumper+wires&amp;qid=1727365183&amp;sprefix=hobby+jumper+wires%2Caps%2C86&amp;sr=8-1-spons&amp;sp_csd=d2lkZ2V0TmFtZT1zcF9hdGY&amp;psc=1" xr:uid="{7F6539C9-5FD8-4849-8F1A-5D2D4B3E252A}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>